<commit_message>
Day 11: SUMIF, AVERAGEIF, COUNTIF and Attendance Tracker
</commit_message>
<xml_diff>
--- a/Excel/Day 10/Excel-Practice-(Day-10).xlsx
+++ b/Excel/Day 10/Excel-Practice-(Day-10).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analyst\Excel\Day 10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E27FCBC-5FFD-41BE-9D76-ECCFCCDA7538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AD6184-28C7-4837-89AC-7711830F006C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="678" firstSheet="19" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5880" yWindow="3450" windowWidth="21600" windowHeight="11835" tabRatio="678" firstSheet="19" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4776" uniqueCount="1205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4824" uniqueCount="1214">
   <si>
     <t>Employee_ID</t>
   </si>
@@ -3318,9 +3318,6 @@
     <t>AGE (datedif)</t>
   </si>
   <si>
-    <t>Meaning (Hinglish)</t>
-  </si>
-  <si>
     <t>IF</t>
   </si>
   <si>
@@ -3706,6 +3703,36 @@
   </si>
   <si>
     <t>GRADE SWITCH</t>
+  </si>
+  <si>
+    <t>IF + TEXT</t>
+  </si>
+  <si>
+    <t>IF(A1&gt;50,"High","Low")</t>
+  </si>
+  <si>
+    <t>Text output decision</t>
+  </si>
+  <si>
+    <t>Reporting</t>
+  </si>
+  <si>
+    <t>Status generation</t>
+  </si>
+  <si>
+    <t>IF + Multiple Conditions</t>
+  </si>
+  <si>
+    <t>IF(A1&gt;90,"A",IF(A1&gt;75,"B",IF(A1&gt;50,"C","Fail")))</t>
+  </si>
+  <si>
+    <t>Multi grading system</t>
+  </si>
+  <si>
+    <t>Education / HR</t>
+  </si>
+  <si>
+    <t>Grade system</t>
   </si>
 </sst>
 </file>
@@ -5937,6 +5964,9 @@
     <xf numFmtId="0" fontId="31" fillId="9" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6048,9 +6078,6 @@
     <xf numFmtId="0" fontId="20" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6074,152 +6101,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="4" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7025,6 +6906,152 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="4" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -7958,15 +7985,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="45" dataDxfId="43" headerRowBorderDxfId="44" tableBorderDxfId="42">
   <autoFilter ref="A1:F38" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="55" totalsRowDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="53" totalsRowDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="51" totalsRowDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="49" totalsRowDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="47" totalsRowDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="44">
+    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
       <totalsRowFormula>SUM(F2:F38)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -20686,22 +20713,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:29" x14ac:dyDescent="0.25">
-      <c r="D1" s="309" t="s">
+      <c r="D1" s="310" t="s">
         <v>541</v>
       </c>
-      <c r="E1" s="310"/>
-      <c r="F1" s="310"/>
-      <c r="G1" s="310"/>
-      <c r="H1" s="310"/>
-      <c r="I1" s="310"/>
-      <c r="X1" s="311" t="s">
+      <c r="E1" s="311"/>
+      <c r="F1" s="311"/>
+      <c r="G1" s="311"/>
+      <c r="H1" s="311"/>
+      <c r="I1" s="311"/>
+      <c r="X1" s="312" t="s">
         <v>542</v>
       </c>
-      <c r="Y1" s="312"/>
-      <c r="Z1" s="312"/>
-      <c r="AA1" s="312"/>
-      <c r="AB1" s="312"/>
-      <c r="AC1" s="313"/>
+      <c r="Y1" s="313"/>
+      <c r="Z1" s="313"/>
+      <c r="AA1" s="313"/>
+      <c r="AB1" s="313"/>
+      <c r="AC1" s="314"/>
     </row>
     <row r="2" spans="4:29" x14ac:dyDescent="0.25">
       <c r="D2" s="106" t="s">
@@ -20722,29 +20749,29 @@
       <c r="I2" s="106" t="s">
         <v>537</v>
       </c>
-      <c r="K2" s="311" t="s">
+      <c r="K2" s="312" t="s">
         <v>543</v>
       </c>
-      <c r="L2" s="312"/>
-      <c r="M2" s="312"/>
-      <c r="N2" s="312"/>
-      <c r="O2" s="312"/>
-      <c r="P2" s="312"/>
-      <c r="Q2" s="312"/>
-      <c r="R2" s="312"/>
-      <c r="S2" s="312"/>
-      <c r="T2" s="312"/>
-      <c r="U2" s="312"/>
-      <c r="V2" s="313"/>
-      <c r="X2" s="309" t="str">
+      <c r="L2" s="313"/>
+      <c r="M2" s="313"/>
+      <c r="N2" s="313"/>
+      <c r="O2" s="313"/>
+      <c r="P2" s="313"/>
+      <c r="Q2" s="313"/>
+      <c r="R2" s="313"/>
+      <c r="S2" s="313"/>
+      <c r="T2" s="313"/>
+      <c r="U2" s="313"/>
+      <c r="V2" s="314"/>
+      <c r="X2" s="310" t="str">
         <f t="shared" ref="X2:X17" si="0">D1</f>
         <v>OPERATIONS</v>
       </c>
-      <c r="Y2" s="310"/>
-      <c r="Z2" s="310"/>
-      <c r="AA2" s="310"/>
-      <c r="AB2" s="310"/>
-      <c r="AC2" s="310"/>
+      <c r="Y2" s="311"/>
+      <c r="Z2" s="311"/>
+      <c r="AA2" s="311"/>
+      <c r="AB2" s="311"/>
+      <c r="AC2" s="311"/>
     </row>
     <row r="3" spans="4:29" x14ac:dyDescent="0.25">
       <c r="D3" s="105" t="s">
@@ -20761,7 +20788,7 @@
       </c>
       <c r="H3" s="135">
         <f t="shared" ref="H3:H16" ca="1" si="1">(RANDBETWEEN(10,50))/100</f>
-        <v>0.38</v>
+        <v>0.22</v>
       </c>
       <c r="I3" s="105">
         <v>100</v>
@@ -20806,7 +20833,7 @@
       </c>
       <c r="H4" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.44</v>
+        <v>0.17</v>
       </c>
       <c r="X4" s="105" t="str">
         <f t="shared" si="0"/>
@@ -20826,7 +20853,7 @@
       </c>
       <c r="AB4" s="135">
         <f t="shared" ca="1" si="2"/>
-        <v>0.38</v>
+        <v>0.22</v>
       </c>
       <c r="AC4" s="105">
         <f t="shared" si="2"/>
@@ -20868,7 +20895,7 @@
       </c>
       <c r="AB5" s="135">
         <f t="shared" ref="AB5:AB17" ca="1" si="6">H4</f>
-        <v>0.44</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="6" spans="4:29" x14ac:dyDescent="0.25">
@@ -20886,20 +20913,20 @@
       </c>
       <c r="H6" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.27</v>
-      </c>
-      <c r="L6" s="311" t="s">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="L6" s="312" t="s">
         <v>540</v>
       </c>
-      <c r="M6" s="312"/>
-      <c r="N6" s="312"/>
-      <c r="O6" s="312"/>
-      <c r="P6" s="312"/>
-      <c r="Q6" s="312"/>
-      <c r="R6" s="312"/>
-      <c r="S6" s="312"/>
-      <c r="T6" s="312"/>
-      <c r="U6" s="313"/>
+      <c r="M6" s="313"/>
+      <c r="N6" s="313"/>
+      <c r="O6" s="313"/>
+      <c r="P6" s="313"/>
+      <c r="Q6" s="313"/>
+      <c r="R6" s="313"/>
+      <c r="S6" s="313"/>
+      <c r="T6" s="313"/>
+      <c r="U6" s="314"/>
       <c r="X6" s="105" t="str">
         <f t="shared" si="0"/>
         <v>Muhammad Hamza</v>
@@ -20936,7 +20963,7 @@
       </c>
       <c r="H7" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
       <c r="X7" s="105" t="str">
         <f t="shared" si="0"/>
@@ -20956,7 +20983,7 @@
       </c>
       <c r="AB7" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.27</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="8" spans="4:29" x14ac:dyDescent="0.25">
@@ -20974,7 +21001,7 @@
       </c>
       <c r="H8" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34</v>
+        <v>0.27</v>
       </c>
       <c r="M8" s="105">
         <v>137196</v>
@@ -21000,7 +21027,7 @@
       </c>
       <c r="AB8" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="9" spans="4:29" x14ac:dyDescent="0.25">
@@ -21018,7 +21045,7 @@
       </c>
       <c r="H9" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.4</v>
+        <v>0.44</v>
       </c>
       <c r="M9" s="105">
         <v>64256</v>
@@ -21042,7 +21069,7 @@
       </c>
       <c r="AB9" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.34</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="10" spans="4:29" x14ac:dyDescent="0.25">
@@ -21060,7 +21087,7 @@
       </c>
       <c r="H10" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.43</v>
+        <v>0.24</v>
       </c>
       <c r="M10" s="105">
         <v>137080</v>
@@ -21086,7 +21113,7 @@
       </c>
       <c r="AB10" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.4</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="11" spans="4:29" x14ac:dyDescent="0.25">
@@ -21104,7 +21131,7 @@
       </c>
       <c r="H11" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.17</v>
+        <v>0.35</v>
       </c>
       <c r="M11" s="105">
         <v>95302</v>
@@ -21130,7 +21157,7 @@
       </c>
       <c r="AB11" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.43</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="12" spans="4:29" x14ac:dyDescent="0.25">
@@ -21148,7 +21175,7 @@
       </c>
       <c r="H12" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.31</v>
+        <v>0.4</v>
       </c>
       <c r="M12" s="105">
         <v>68657</v>
@@ -21174,7 +21201,7 @@
       </c>
       <c r="AB12" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.17</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="13" spans="4:29" x14ac:dyDescent="0.25">
@@ -21192,7 +21219,7 @@
       </c>
       <c r="H13" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
       <c r="M13" s="105">
         <v>66062</v>
@@ -21218,7 +21245,7 @@
       </c>
       <c r="AB13" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.31</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14" spans="4:29" x14ac:dyDescent="0.25">
@@ -21236,7 +21263,7 @@
       </c>
       <c r="H14" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="M14" s="105">
         <v>98878</v>
@@ -21262,7 +21289,7 @@
       </c>
       <c r="AB14" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="15" spans="4:29" x14ac:dyDescent="0.25">
@@ -21280,7 +21307,7 @@
       </c>
       <c r="H15" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.27</v>
+        <v>0.46</v>
       </c>
       <c r="M15" s="105">
         <v>40851</v>
@@ -21306,7 +21333,7 @@
       </c>
       <c r="AB15" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="16" spans="4:29" x14ac:dyDescent="0.25">
@@ -21324,7 +21351,7 @@
       </c>
       <c r="H16" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.38</v>
+        <v>0.26</v>
       </c>
       <c r="M16" s="105"/>
       <c r="N16" s="105"/>
@@ -21346,7 +21373,7 @@
       </c>
       <c r="AB16" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.27</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="17" spans="4:28" x14ac:dyDescent="0.25">
@@ -21375,7 +21402,7 @@
       </c>
       <c r="AB17" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.38</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="18" spans="4:28" x14ac:dyDescent="0.25">
@@ -21423,31 +21450,31 @@
       </c>
     </row>
     <row r="29" spans="4:28" x14ac:dyDescent="0.25">
-      <c r="D29" s="310" t="s">
+      <c r="D29" s="311" t="s">
         <v>538</v>
       </c>
-      <c r="E29" s="310"/>
-      <c r="F29" s="310"/>
-      <c r="G29" s="310"/>
-      <c r="H29" s="310"/>
-      <c r="I29" s="310"/>
-      <c r="J29" s="310"/>
-      <c r="K29" s="310"/>
-      <c r="L29" s="310"/>
-      <c r="M29" s="310"/>
-      <c r="N29" s="310"/>
-      <c r="O29" s="310"/>
-      <c r="P29" s="310"/>
-      <c r="Q29" s="310"/>
-      <c r="R29" s="310"/>
-      <c r="U29" s="311" t="s">
+      <c r="E29" s="311"/>
+      <c r="F29" s="311"/>
+      <c r="G29" s="311"/>
+      <c r="H29" s="311"/>
+      <c r="I29" s="311"/>
+      <c r="J29" s="311"/>
+      <c r="K29" s="311"/>
+      <c r="L29" s="311"/>
+      <c r="M29" s="311"/>
+      <c r="N29" s="311"/>
+      <c r="O29" s="311"/>
+      <c r="P29" s="311"/>
+      <c r="Q29" s="311"/>
+      <c r="R29" s="311"/>
+      <c r="U29" s="312" t="s">
         <v>539</v>
       </c>
-      <c r="V29" s="312"/>
-      <c r="W29" s="312"/>
-      <c r="X29" s="312"/>
-      <c r="Y29" s="312"/>
-      <c r="Z29" s="313"/>
+      <c r="V29" s="313"/>
+      <c r="W29" s="313"/>
+      <c r="X29" s="313"/>
+      <c r="Y29" s="313"/>
+      <c r="Z29" s="314"/>
     </row>
     <row r="30" spans="4:28" x14ac:dyDescent="0.25">
       <c r="D30" s="106" t="s">
@@ -21991,38 +22018,38 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A4" s="314" t="s">
+      <c r="A4" s="315" t="s">
         <v>545</v>
       </c>
-      <c r="B4" s="315"/>
-      <c r="C4" s="315"/>
-      <c r="D4" s="315"/>
-      <c r="E4" s="315"/>
-      <c r="F4" s="315"/>
-      <c r="H4" s="314" t="s">
+      <c r="B4" s="316"/>
+      <c r="C4" s="316"/>
+      <c r="D4" s="316"/>
+      <c r="E4" s="316"/>
+      <c r="F4" s="316"/>
+      <c r="H4" s="315" t="s">
         <v>546</v>
       </c>
-      <c r="I4" s="315"/>
-      <c r="J4" s="315"/>
-      <c r="K4" s="315"/>
-      <c r="L4" s="315"/>
-      <c r="M4" s="315"/>
-      <c r="P4" s="314" t="s">
+      <c r="I4" s="316"/>
+      <c r="J4" s="316"/>
+      <c r="K4" s="316"/>
+      <c r="L4" s="316"/>
+      <c r="M4" s="316"/>
+      <c r="P4" s="315" t="s">
         <v>548</v>
       </c>
-      <c r="Q4" s="315"/>
-      <c r="R4" s="315"/>
-      <c r="S4" s="315"/>
-      <c r="T4" s="315"/>
-      <c r="U4" s="315"/>
-      <c r="W4" s="314" t="s">
+      <c r="Q4" s="316"/>
+      <c r="R4" s="316"/>
+      <c r="S4" s="316"/>
+      <c r="T4" s="316"/>
+      <c r="U4" s="316"/>
+      <c r="W4" s="315" t="s">
         <v>547</v>
       </c>
-      <c r="X4" s="315"/>
-      <c r="Y4" s="315"/>
-      <c r="Z4" s="315"/>
-      <c r="AA4" s="315"/>
-      <c r="AB4" s="315"/>
+      <c r="X4" s="316"/>
+      <c r="Y4" s="316"/>
+      <c r="Z4" s="316"/>
+      <c r="AA4" s="316"/>
+      <c r="AB4" s="316"/>
     </row>
     <row r="5" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
@@ -24491,22 +24518,22 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="316" t="s">
+      <c r="B3" s="317" t="s">
         <v>553</v>
       </c>
-      <c r="C3" s="316"/>
-      <c r="D3" s="316"/>
-      <c r="E3" s="316"/>
-      <c r="F3" s="316"/>
-      <c r="G3" s="317">
+      <c r="C3" s="317"/>
+      <c r="D3" s="317"/>
+      <c r="E3" s="317"/>
+      <c r="F3" s="317"/>
+      <c r="G3" s="318">
         <v>400</v>
       </c>
-      <c r="H3" s="317"/>
-      <c r="I3" s="317"/>
-      <c r="J3" s="317"/>
-      <c r="K3" s="317"/>
-      <c r="L3" s="317"/>
-      <c r="M3" s="317"/>
+      <c r="H3" s="318"/>
+      <c r="I3" s="318"/>
+      <c r="J3" s="318"/>
+      <c r="K3" s="318"/>
+      <c r="L3" s="318"/>
+      <c r="M3" s="318"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="137" t="s">
@@ -25207,18 +25234,18 @@
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B25" s="316" t="s">
+      <c r="B25" s="317" t="s">
         <v>553</v>
       </c>
-      <c r="C25" s="316"/>
-      <c r="D25" s="316"/>
-      <c r="E25" s="316"/>
-      <c r="F25" s="316"/>
-      <c r="G25" s="318">
+      <c r="C25" s="317"/>
+      <c r="D25" s="317"/>
+      <c r="E25" s="317"/>
+      <c r="F25" s="317"/>
+      <c r="G25" s="319">
         <v>400</v>
       </c>
-      <c r="H25" s="319"/>
-      <c r="I25" s="319"/>
+      <c r="H25" s="320"/>
+      <c r="I25" s="320"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="137" t="s">
@@ -26112,14 +26139,14 @@
       </c>
     </row>
     <row r="24" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="320" t="s">
+      <c r="B24" s="321" t="s">
         <v>734</v>
       </c>
-      <c r="C24" s="321"/>
-      <c r="D24" s="321"/>
-      <c r="E24" s="321"/>
-      <c r="F24" s="321"/>
-      <c r="G24" s="322"/>
+      <c r="C24" s="322"/>
+      <c r="D24" s="322"/>
+      <c r="E24" s="322"/>
+      <c r="F24" s="322"/>
+      <c r="G24" s="323"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="G31" s="238"/>
@@ -26164,19 +26191,19 @@
   <sheetData>
     <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="323" t="s">
+      <c r="B2" s="324" t="s">
         <v>564</v>
       </c>
-      <c r="C2" s="324"/>
+      <c r="C2" s="325"/>
       <c r="D2" s="145"/>
-      <c r="E2" s="323" t="s">
+      <c r="E2" s="324" t="s">
         <v>568</v>
       </c>
-      <c r="F2" s="324"/>
-      <c r="H2" s="323" t="s">
+      <c r="F2" s="325"/>
+      <c r="H2" s="324" t="s">
         <v>572</v>
       </c>
-      <c r="I2" s="324"/>
+      <c r="I2" s="325"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="148" t="s">
@@ -26417,14 +26444,14 @@
     </row>
     <row r="15" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="323" t="s">
+      <c r="B16" s="324" t="s">
         <v>687</v>
       </c>
-      <c r="C16" s="324"/>
-      <c r="E16" s="323" t="s">
+      <c r="C16" s="325"/>
+      <c r="E16" s="324" t="s">
         <v>580</v>
       </c>
-      <c r="F16" s="324"/>
+      <c r="F16" s="325"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="148" t="s">
@@ -26582,18 +26609,18 @@
     </row>
     <row r="31" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="323" t="s">
+      <c r="B32" s="324" t="s">
         <v>588</v>
       </c>
-      <c r="C32" s="324"/>
-      <c r="E32" s="323" t="s">
+      <c r="C32" s="325"/>
+      <c r="E32" s="324" t="s">
         <v>584</v>
       </c>
-      <c r="F32" s="324"/>
-      <c r="H32" s="323" t="s">
+      <c r="F32" s="325"/>
+      <c r="H32" s="324" t="s">
         <v>592</v>
       </c>
-      <c r="I32" s="324"/>
+      <c r="I32" s="325"/>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B33" s="148" t="s">
@@ -26823,39 +26850,39 @@
       </c>
     </row>
     <row r="45" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="325" t="s">
+      <c r="B45" s="326" t="s">
         <v>732</v>
       </c>
-      <c r="C45" s="325"/>
-      <c r="D45" s="325"/>
+      <c r="C45" s="326"/>
+      <c r="D45" s="326"/>
       <c r="E45" s="170"/>
       <c r="F45" s="170"/>
-      <c r="G45" s="325" t="s">
+      <c r="G45" s="326" t="s">
         <v>719</v>
       </c>
-      <c r="H45" s="325"/>
-      <c r="I45" s="325"/>
+      <c r="H45" s="326"/>
+      <c r="I45" s="326"/>
       <c r="J45" s="170"/>
-      <c r="K45" s="325" t="s">
+      <c r="K45" s="326" t="s">
         <v>707</v>
       </c>
-      <c r="L45" s="325"/>
-      <c r="M45" s="325"/>
-      <c r="O45" s="325" t="s">
+      <c r="L45" s="326"/>
+      <c r="M45" s="326"/>
+      <c r="O45" s="326" t="s">
         <v>730</v>
       </c>
-      <c r="P45" s="325"/>
-      <c r="Q45" s="325"/>
-      <c r="S45" s="325" t="s">
+      <c r="P45" s="326"/>
+      <c r="Q45" s="326"/>
+      <c r="S45" s="326" t="s">
         <v>731</v>
       </c>
-      <c r="T45" s="325"/>
-      <c r="U45" s="325"/>
-      <c r="W45" s="325" t="s">
+      <c r="T45" s="326"/>
+      <c r="U45" s="326"/>
+      <c r="W45" s="326" t="s">
         <v>733</v>
       </c>
-      <c r="X45" s="325"/>
-      <c r="Y45" s="325"/>
+      <c r="X45" s="326"/>
+      <c r="Y45" s="326"/>
     </row>
     <row r="46" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="167" t="s">
@@ -27542,11 +27569,11 @@
       <c r="D59" s="170"/>
       <c r="E59" s="170"/>
       <c r="F59" s="170"/>
-      <c r="G59" s="325" t="s">
+      <c r="G59" s="326" t="s">
         <v>735</v>
       </c>
-      <c r="H59" s="325"/>
-      <c r="I59" s="325"/>
+      <c r="H59" s="326"/>
+      <c r="I59" s="326"/>
       <c r="J59" s="170"/>
       <c r="K59" s="170"/>
       <c r="L59" s="170"/>
@@ -27653,22 +27680,22 @@
     </row>
     <row r="74" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="75" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B75" s="323" t="s">
+      <c r="B75" s="324" t="s">
         <v>738</v>
       </c>
-      <c r="C75" s="324"/>
-      <c r="E75" s="323" t="s">
+      <c r="C75" s="325"/>
+      <c r="E75" s="324" t="s">
         <v>741</v>
       </c>
-      <c r="F75" s="324"/>
-      <c r="H75" s="323" t="s">
+      <c r="F75" s="325"/>
+      <c r="H75" s="324" t="s">
         <v>740</v>
       </c>
-      <c r="I75" s="324"/>
-      <c r="K75" s="323" t="s">
+      <c r="I75" s="325"/>
+      <c r="K75" s="324" t="s">
         <v>742</v>
       </c>
-      <c r="L75" s="324"/>
+      <c r="L75" s="325"/>
     </row>
     <row r="76" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B76" s="148" t="s">
@@ -27968,10 +27995,10 @@
     </row>
     <row r="89" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="90" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="323" t="s">
+      <c r="B90" s="324" t="s">
         <v>628</v>
       </c>
-      <c r="C90" s="324"/>
+      <c r="C90" s="325"/>
     </row>
     <row r="91" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B91" s="148" t="s">
@@ -27983,14 +28010,14 @@
       <c r="D91" s="148" t="s">
         <v>745</v>
       </c>
-      <c r="F91" s="323" t="s">
+      <c r="F91" s="324" t="s">
         <v>746</v>
       </c>
-      <c r="G91" s="324"/>
-      <c r="I91" s="323" t="s">
+      <c r="G91" s="325"/>
+      <c r="I91" s="324" t="s">
         <v>748</v>
       </c>
-      <c r="J91" s="324"/>
+      <c r="J91" s="325"/>
     </row>
     <row r="92" spans="2:12" ht="30" x14ac:dyDescent="0.25">
       <c r="B92" s="183">
@@ -28083,14 +28110,14 @@
         <f t="shared" si="17"/>
         <v>October</v>
       </c>
-      <c r="F97" s="323" t="s">
+      <c r="F97" s="324" t="s">
         <v>637</v>
       </c>
-      <c r="G97" s="324"/>
-      <c r="I97" s="323" t="s">
+      <c r="G97" s="325"/>
+      <c r="I97" s="324" t="s">
         <v>641</v>
       </c>
-      <c r="J97" s="324"/>
+      <c r="J97" s="325"/>
     </row>
     <row r="98" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B98" s="183">
@@ -28147,6 +28174,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="H75:I75"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="I91:J91"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="E16:F16"/>
     <mergeCell ref="F97:G97"/>
     <mergeCell ref="I97:J97"/>
     <mergeCell ref="W45:Y45"/>
@@ -28163,14 +28198,6 @@
     <mergeCell ref="B75:C75"/>
     <mergeCell ref="E75:F75"/>
     <mergeCell ref="K75:L75"/>
-    <mergeCell ref="H75:I75"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="I91:J91"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="E16:F16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -28813,14 +28840,14 @@
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="326" t="s">
+      <c r="B34" s="327" t="s">
         <v>898</v>
       </c>
-      <c r="C34" s="327"/>
-      <c r="D34" s="327"/>
-      <c r="E34" s="327"/>
-      <c r="F34" s="327"/>
-      <c r="G34" s="328"/>
+      <c r="C34" s="328"/>
+      <c r="D34" s="328"/>
+      <c r="E34" s="328"/>
+      <c r="F34" s="328"/>
+      <c r="G34" s="329"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -28856,29 +28883,29 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="329" t="s">
+      <c r="B3" s="330" t="s">
         <v>899</v>
       </c>
-      <c r="C3" s="329"/>
-      <c r="D3" s="329"/>
-      <c r="F3" s="325" t="s">
+      <c r="C3" s="330"/>
+      <c r="D3" s="330"/>
+      <c r="F3" s="326" t="s">
         <v>828</v>
       </c>
-      <c r="G3" s="325"/>
-      <c r="H3" s="325"/>
+      <c r="G3" s="326"/>
+      <c r="H3" s="326"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4" s="209">
         <f t="shared" ref="B4:D13" ca="1" si="0">RAND()</f>
-        <v>0.60377537416444638</v>
+        <v>0.28840726126944494</v>
       </c>
       <c r="C4" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.23450436042729994</v>
+        <v>0.67576056450093569</v>
       </c>
       <c r="D4" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.54380795295214623</v>
+        <v>0.74721517123265413</v>
       </c>
       <c r="F4" s="167" t="s">
         <v>901</v>
@@ -28893,15 +28920,15 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.97535827797783115</v>
+        <v>0.78396109618356258</v>
       </c>
       <c r="C5" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>6.0402949682730966E-2</v>
+        <v>0.54380393483457667</v>
       </c>
       <c r="D5" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.90209114338025576</v>
+        <v>0.75549825329508136</v>
       </c>
       <c r="F5" s="169">
         <v>1</v>
@@ -28917,15 +28944,15 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.50256991049618749</v>
+        <v>0.68706239228534172</v>
       </c>
       <c r="C6" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.10351338527281784</v>
+        <v>0.68477649227830728</v>
       </c>
       <c r="D6" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.24847111971147229</v>
+        <v>0.90928519966158661</v>
       </c>
       <c r="F6" s="169">
         <v>2</v>
@@ -28941,15 +28968,15 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.74102219654330492</v>
+        <v>0.38405589329927592</v>
       </c>
       <c r="C7" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.35724414348420341</v>
+        <v>0.65762555107116283</v>
       </c>
       <c r="D7" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.29122662501999075</v>
+        <v>0.70322120693574663</v>
       </c>
       <c r="F7" s="169">
         <v>3</v>
@@ -28965,15 +28992,15 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.11059133178825986</v>
+        <v>0.86594197581878585</v>
       </c>
       <c r="C8" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.82971642592236927</v>
+        <v>0.93508456035653309</v>
       </c>
       <c r="D8" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.45149796311619383</v>
+        <v>0.81173866207228795</v>
       </c>
       <c r="F8" s="169">
         <v>4</v>
@@ -28989,15 +29016,15 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B9" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.69304118568209516</v>
+        <v>0.3173712203446406</v>
       </c>
       <c r="C9" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.65843493518685159</v>
+        <v>0.27975171808764876</v>
       </c>
       <c r="D9" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.2478571362353551</v>
+        <v>0.34927261649475083</v>
       </c>
       <c r="F9" s="169">
         <v>5</v>
@@ -29013,15 +29040,15 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.40672179928189367</v>
+        <v>0.17982078986140582</v>
       </c>
       <c r="C10" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84164521365856149</v>
+        <v>1.6784089641795785E-2</v>
       </c>
       <c r="D10" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>3.1686609225126783E-2</v>
+        <v>0.23286147564128279</v>
       </c>
       <c r="F10" s="169">
         <v>6</v>
@@ -29037,15 +29064,15 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.28238064992972911</v>
+        <v>0.5445730731149161</v>
       </c>
       <c r="C11" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84049920140311973</v>
+        <v>0.65177395273201544</v>
       </c>
       <c r="D11" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.63848014481677162</v>
+        <v>0.46730631268962797</v>
       </c>
       <c r="F11" s="169">
         <v>7</v>
@@ -29061,15 +29088,15 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>1.9727056569237567E-3</v>
+        <v>0.41325000552988245</v>
       </c>
       <c r="C12" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.46971506843669875</v>
+        <v>0.35210904602577331</v>
       </c>
       <c r="D12" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.40185599771245384</v>
+        <v>0.38977265732622579</v>
       </c>
       <c r="F12" s="169">
         <v>8</v>
@@ -29085,15 +29112,15 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B13" s="209">
         <f t="shared" ca="1" si="0"/>
-        <v>0.41096487441273577</v>
+        <v>0.77819541283637439</v>
       </c>
       <c r="C13" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.74725112816684802</v>
+        <v>0.31984341634601332</v>
       </c>
       <c r="D13" s="168">
         <f t="shared" ca="1" si="0"/>
-        <v>0.99528249142563463</v>
+        <v>4.9989435984913011E-2</v>
       </c>
       <c r="F13" s="169">
         <v>9</v>
@@ -29119,35 +29146,35 @@
       </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="330" t="s">
+      <c r="B17" s="331" t="s">
         <v>900</v>
       </c>
-      <c r="C17" s="329"/>
-      <c r="D17" s="329"/>
-      <c r="F17" s="325" t="s">
+      <c r="C17" s="330"/>
+      <c r="D17" s="330"/>
+      <c r="F17" s="326" t="s">
         <v>903</v>
       </c>
-      <c r="G17" s="325"/>
-      <c r="H17" s="325"/>
-      <c r="J17" s="325" t="s">
+      <c r="G17" s="326"/>
+      <c r="H17" s="326"/>
+      <c r="J17" s="326" t="s">
         <v>906</v>
       </c>
-      <c r="K17" s="325"/>
-      <c r="L17" s="325"/>
-      <c r="M17" s="325"/>
+      <c r="K17" s="326"/>
+      <c r="L17" s="326"/>
+      <c r="M17" s="326"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="209">
         <f ca="1">RANDBETWEEN(0,100)</f>
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="C18" s="168">
         <f t="shared" ref="B18:D27" ca="1" si="2">RANDBETWEEN(0,100)</f>
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="D18" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F18" s="167" t="s">
         <v>901</v>
@@ -29174,15 +29201,15 @@
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="C19" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="D19" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="F19" s="169">
         <v>1</v>
@@ -29212,15 +29239,15 @@
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C20" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D20" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="F20" s="169">
         <v>2</v>
@@ -29250,15 +29277,15 @@
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="C21" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="D21" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="F21" s="169">
         <v>3</v>
@@ -29288,15 +29315,15 @@
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="C22" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="D22" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>93</v>
+        <v>21</v>
       </c>
       <c r="F22" s="169">
         <v>4</v>
@@ -29326,15 +29353,15 @@
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>88</v>
       </c>
       <c r="C23" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="D23" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="F23" s="169">
         <v>5</v>
@@ -29364,15 +29391,15 @@
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="C24" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D24" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="F24" s="169">
         <v>6</v>
@@ -29402,15 +29429,15 @@
     <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="C25" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="D25" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="F25" s="169">
         <v>7</v>
@@ -29440,15 +29467,15 @@
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="C26" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D26" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="F26" s="169">
         <v>8</v>
@@ -29478,15 +29505,15 @@
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="209">
         <f t="shared" ca="1" si="2"/>
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="C27" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="D27" s="168">
         <f t="shared" ca="1" si="2"/>
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="F27" s="169">
         <v>9</v>
@@ -29540,29 +29567,29 @@
       </c>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="329" t="s">
+      <c r="B30" s="330" t="s">
         <v>873</v>
       </c>
-      <c r="C30" s="329"/>
-      <c r="D30" s="329"/>
-      <c r="F30" s="325" t="s">
+      <c r="C30" s="330"/>
+      <c r="D30" s="330"/>
+      <c r="F30" s="326" t="s">
         <v>904</v>
       </c>
-      <c r="G30" s="325"/>
-      <c r="H30" s="325"/>
+      <c r="G30" s="326"/>
+      <c r="H30" s="326"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B31" s="209" cm="1">
         <f t="array" aca="1" ref="B31:D40" ca="1">_xlfn.RANDARRAY(10,3,0,100,TRUE)</f>
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="C31" s="168">
         <f ca="1"/>
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="D31" s="168">
         <f ca="1"/>
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="F31" s="167" t="s">
         <v>901</v>
@@ -29573,26 +29600,26 @@
       <c r="H31" s="167" t="s">
         <v>904</v>
       </c>
-      <c r="J31" s="325" t="s">
+      <c r="J31" s="326" t="s">
         <v>912</v>
       </c>
-      <c r="K31" s="325"/>
-      <c r="L31" s="325"/>
-      <c r="M31" s="325"/>
-      <c r="N31" s="325"/>
+      <c r="K31" s="326"/>
+      <c r="L31" s="326"/>
+      <c r="M31" s="326"/>
+      <c r="N31" s="326"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B32" s="209">
         <f ca="1"/>
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="C32" s="168">
         <f ca="1"/>
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D32" s="168">
         <f ca="1"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F32" s="169">
         <v>1</v>
@@ -29627,11 +29654,11 @@
       </c>
       <c r="C33" s="168">
         <f ca="1"/>
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D33" s="168">
         <f ca="1"/>
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="F33" s="169">
         <v>2</v>
@@ -29665,15 +29692,15 @@
     <row r="34" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B34" s="209">
         <f ca="1"/>
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="C34" s="168">
         <f ca="1"/>
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="D34" s="168">
         <f ca="1"/>
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="F34" s="169">
         <v>3</v>
@@ -29707,15 +29734,15 @@
     <row r="35" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B35" s="209">
         <f ca="1"/>
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="C35" s="168">
         <f ca="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="D35" s="168">
         <f ca="1"/>
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="F35" s="169">
         <v>4</v>
@@ -29749,15 +29776,15 @@
     <row r="36" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B36" s="209">
         <f ca="1"/>
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="C36" s="168">
         <f ca="1"/>
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="D36" s="168">
         <f ca="1"/>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F36" s="169">
         <v>5</v>
@@ -29791,15 +29818,15 @@
     <row r="37" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B37" s="209">
         <f ca="1"/>
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="C37" s="168">
         <f ca="1"/>
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="D37" s="168">
         <f ca="1"/>
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F37" s="169">
         <v>6</v>
@@ -29833,15 +29860,15 @@
     <row r="38" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B38" s="209">
         <f ca="1"/>
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="C38" s="168">
         <f ca="1"/>
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D38" s="168">
         <f ca="1"/>
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="F38" s="169">
         <v>7</v>
@@ -29875,15 +29902,15 @@
     <row r="39" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B39" s="209">
         <f ca="1"/>
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C39" s="168">
         <f ca="1"/>
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="D39" s="168">
         <f ca="1"/>
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="F39" s="169">
         <v>8</v>
@@ -29917,15 +29944,15 @@
     <row r="40" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B40" s="209">
         <f ca="1"/>
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="C40" s="168">
         <f ca="1"/>
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="D40" s="168">
         <f ca="1"/>
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="F40" s="169">
         <v>9</v>
@@ -30007,16 +30034,16 @@
       </c>
     </row>
     <row r="43" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B43" s="325" t="s">
+      <c r="B43" s="326" t="s">
         <v>813</v>
       </c>
-      <c r="C43" s="325"/>
-      <c r="D43" s="325"/>
-      <c r="F43" s="325" t="s">
+      <c r="C43" s="326"/>
+      <c r="D43" s="326"/>
+      <c r="F43" s="326" t="s">
         <v>818</v>
       </c>
-      <c r="G43" s="325"/>
-      <c r="H43" s="325"/>
+      <c r="G43" s="326"/>
+      <c r="H43" s="326"/>
     </row>
     <row r="44" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B44" s="167" t="s">
@@ -30058,15 +30085,15 @@
         <f t="array" ref="H45:H54">SMALL($G$45:$G$54,F45:F54)</f>
         <v>128</v>
       </c>
-      <c r="J45" s="325" t="s">
+      <c r="J45" s="326" t="s">
         <v>913</v>
       </c>
-      <c r="K45" s="325"/>
-      <c r="L45" s="325"/>
-      <c r="M45" s="325"/>
-      <c r="N45" s="325"/>
-      <c r="O45" s="325"/>
-      <c r="P45" s="325"/>
+      <c r="K45" s="326"/>
+      <c r="L45" s="326"/>
+      <c r="M45" s="326"/>
+      <c r="N45" s="326"/>
+      <c r="O45" s="326"/>
+      <c r="P45" s="326"/>
     </row>
     <row r="46" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B46" s="169">
@@ -31152,14 +31179,14 @@
       </c>
     </row>
     <row r="32" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="331" t="s">
+      <c r="B32" s="332" t="s">
         <v>1047</v>
       </c>
-      <c r="C32" s="332"/>
-      <c r="D32" s="332"/>
-      <c r="E32" s="332"/>
-      <c r="F32" s="332"/>
-      <c r="G32" s="333"/>
+      <c r="C32" s="333"/>
+      <c r="D32" s="333"/>
+      <c r="E32" s="333"/>
+      <c r="F32" s="333"/>
+      <c r="G32" s="334"/>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="246"/>
@@ -31208,7 +31235,7 @@
       </c>
       <c r="D4" s="273" t="str">
         <f ca="1">TEXT(TODAY(), "mm-dd-yyyy")</f>
-        <v>10-19-2026</v>
+        <v>10-20-2026</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -31220,7 +31247,7 @@
       </c>
       <c r="D5" s="273" t="str">
         <f ca="1">TEXT(NOW()+7, "h:mm:ss AM/PM")</f>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -31230,7 +31257,7 @@
       <c r="C6" s="274"/>
       <c r="D6" s="273" t="str">
         <f ca="1">TEXT(NOW() + (7/24), "h:mm:ss AM/PM")</f>
-        <v>6:45:30 AM</v>
+        <v>1:09:48 AM</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -31728,19 +31755,19 @@
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="254" t="str">
         <f ca="1">TEXT(NOW(), "h:mm:ss AM/PM")</f>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C32" s="275">
         <f ca="1">HOUR(B32)</f>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D32" s="275">
         <f ca="1">MINUTE(B32)</f>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E32" s="275">
         <f ca="1">SECOND(B32)</f>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F32" s="275" t="str">
         <f t="shared" ref="F32:F49" si="5">TEXT(A1,"AM/PM")</f>
@@ -31748,25 +31775,25 @@
       </c>
       <c r="G32" s="277">
         <f t="shared" ref="G32:G49" ca="1" si="6">TIME(C32,D32,E32)</f>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="254" t="str">
         <f t="shared" ref="B33:B49" ca="1" si="7">TEXT(NOW(), "h:mm:ss AM/PM")</f>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C33" s="275">
         <f t="shared" ref="C33:C49" ca="1" si="8">HOUR(B33)</f>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D33" s="275">
         <f t="shared" ref="D33:D49" ca="1" si="9">MINUTE(B33)</f>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E33" s="275">
         <f t="shared" ref="E33:E49" ca="1" si="10">SECOND(B33)</f>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F33" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31774,25 +31801,25 @@
       </c>
       <c r="G33" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C34" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D34" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E34" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F34" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31800,25 +31827,25 @@
       </c>
       <c r="G34" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C35" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D35" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E35" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F35" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31826,25 +31853,25 @@
       </c>
       <c r="G35" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C36" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D36" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E36" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F36" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31852,25 +31879,25 @@
       </c>
       <c r="G36" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C37" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D37" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E37" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F37" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31878,25 +31905,25 @@
       </c>
       <c r="G37" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B38" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C38" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D38" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E38" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F38" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31904,25 +31931,25 @@
       </c>
       <c r="G38" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B39" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C39" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D39" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E39" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F39" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31930,25 +31957,25 @@
       </c>
       <c r="G39" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C40" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D40" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E40" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F40" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31956,25 +31983,25 @@
       </c>
       <c r="G40" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B41" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C41" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D41" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E41" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F41" s="275" t="str">
         <f t="shared" si="5"/>
@@ -31982,25 +32009,25 @@
       </c>
       <c r="G41" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B42" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C42" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D42" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E42" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F42" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32008,25 +32035,25 @@
       </c>
       <c r="G42" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C43" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D43" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E43" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F43" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32034,25 +32061,25 @@
       </c>
       <c r="G43" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C44" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D44" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E44" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F44" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32060,25 +32087,25 @@
       </c>
       <c r="G44" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B45" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C45" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D45" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E45" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F45" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32086,25 +32113,25 @@
       </c>
       <c r="G45" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B46" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C46" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D46" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E46" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F46" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32112,25 +32139,25 @@
       </c>
       <c r="G46" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B47" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C47" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D47" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E47" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F47" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32138,25 +32165,25 @@
       </c>
       <c r="G47" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B48" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C48" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D48" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E48" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F48" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32164,25 +32191,25 @@
       </c>
       <c r="G48" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B49" s="254" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>11:45:30 PM</v>
+        <v>6:09:48 PM</v>
       </c>
       <c r="C49" s="275">
         <f t="shared" ca="1" si="8"/>
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D49" s="275">
         <f t="shared" ca="1" si="9"/>
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E49" s="275">
         <f t="shared" ca="1" si="10"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F49" s="275" t="str">
         <f t="shared" si="5"/>
@@ -32190,7 +32217,7 @@
       </c>
       <c r="G49" s="277">
         <f t="shared" ca="1" si="6"/>
-        <v>0.98993055555555554</v>
+        <v>0.75680555555555551</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -33698,7 +33725,7 @@
       </c>
       <c r="C119" s="291" t="str">
         <f ca="1">TEXT(NOW(),"MM-DD-YYYY")</f>
-        <v>10-19-2026</v>
+        <v>10-20-2026</v>
       </c>
       <c r="D119" s="293">
         <f ca="1">DATEDIF(B119,C119,"Y")</f>
@@ -33706,7 +33733,7 @@
       </c>
       <c r="E119" s="293">
         <f ca="1">YEARFRAC(B119,C119)</f>
-        <v>21.958333333333332</v>
+        <v>21.961111111111112</v>
       </c>
     </row>
     <row r="120" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -33715,7 +33742,7 @@
       </c>
       <c r="C120" s="291" t="str">
         <f ca="1">TEXT(NOW(),"MM-DD-YYYY")</f>
-        <v>10-19-2026</v>
+        <v>10-20-2026</v>
       </c>
       <c r="D120" s="293">
         <f ca="1">DATEDIF(B120,C120,"Y")</f>
@@ -33723,7 +33750,7 @@
       </c>
       <c r="E120" s="293">
         <f ca="1">YEARFRAC(B120,C120)</f>
-        <v>20.927777777777777</v>
+        <v>20.930555555555557</v>
       </c>
     </row>
   </sheetData>
@@ -36139,7 +36166,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE363568-819E-490C-9224-94253261D52F}">
-  <dimension ref="C6:H26"/>
+  <dimension ref="C6:H40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
@@ -36161,7 +36188,7 @@
         <v>561</v>
       </c>
       <c r="F6" s="239" t="s">
-        <v>1075</v>
+        <v>645</v>
       </c>
       <c r="G6" s="239" t="s">
         <v>562</v>
@@ -36175,19 +36202,19 @@
         <v>1</v>
       </c>
       <c r="D7" s="294" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E7" s="240" t="s">
         <v>1076</v>
       </c>
-      <c r="E7" s="240" t="s">
+      <c r="F7" s="240" t="s">
         <v>1077</v>
       </c>
-      <c r="F7" s="240" t="s">
+      <c r="G7" s="240" t="s">
         <v>1078</v>
       </c>
-      <c r="G7" s="240" t="s">
+      <c r="H7" s="240" t="s">
         <v>1079</v>
-      </c>
-      <c r="H7" s="240" t="s">
-        <v>1080</v>
       </c>
     </row>
     <row r="8" spans="3:8" x14ac:dyDescent="0.25">
@@ -36195,19 +36222,19 @@
         <v>2</v>
       </c>
       <c r="D8" s="294" t="s">
+        <v>1080</v>
+      </c>
+      <c r="E8" s="240" t="s">
         <v>1081</v>
       </c>
-      <c r="E8" s="240" t="s">
+      <c r="F8" s="240" t="s">
         <v>1082</v>
       </c>
-      <c r="F8" s="240" t="s">
+      <c r="G8" s="240" t="s">
         <v>1083</v>
       </c>
-      <c r="G8" s="240" t="s">
+      <c r="H8" s="240" t="s">
         <v>1084</v>
-      </c>
-      <c r="H8" s="240" t="s">
-        <v>1085</v>
       </c>
     </row>
     <row r="9" spans="3:8" x14ac:dyDescent="0.25">
@@ -36215,16 +36242,16 @@
         <v>3</v>
       </c>
       <c r="D9" s="295" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E9" s="249" t="s">
         <v>1086</v>
       </c>
-      <c r="E9" s="249" t="s">
+      <c r="F9" s="249" t="s">
         <v>1087</v>
       </c>
-      <c r="F9" s="249" t="s">
+      <c r="G9" s="249" t="s">
         <v>1088</v>
-      </c>
-      <c r="G9" s="249" t="s">
-        <v>1089</v>
       </c>
       <c r="H9" s="249" t="b">
         <v>0</v>
@@ -36235,16 +36262,16 @@
         <v>4</v>
       </c>
       <c r="D10" s="295" t="s">
+        <v>1089</v>
+      </c>
+      <c r="E10" s="249" t="s">
         <v>1090</v>
       </c>
-      <c r="E10" s="249" t="s">
+      <c r="F10" s="249" t="s">
         <v>1091</v>
       </c>
-      <c r="F10" s="249" t="s">
+      <c r="G10" s="249" t="s">
         <v>1092</v>
-      </c>
-      <c r="G10" s="249" t="s">
-        <v>1093</v>
       </c>
       <c r="H10" s="249" t="b">
         <v>1</v>
@@ -36255,16 +36282,16 @@
         <v>5</v>
       </c>
       <c r="D11" s="295" t="s">
+        <v>1093</v>
+      </c>
+      <c r="E11" s="249" t="s">
         <v>1094</v>
       </c>
-      <c r="E11" s="249" t="s">
+      <c r="F11" s="249" t="s">
         <v>1095</v>
       </c>
-      <c r="F11" s="249" t="s">
+      <c r="G11" s="249" t="s">
         <v>1096</v>
-      </c>
-      <c r="G11" s="249" t="s">
-        <v>1097</v>
       </c>
       <c r="H11" s="249" t="b">
         <v>0</v>
@@ -36275,19 +36302,19 @@
         <v>6</v>
       </c>
       <c r="D12" s="295" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E12" s="249" t="s">
         <v>1098</v>
       </c>
-      <c r="E12" s="249" t="s">
+      <c r="F12" s="249" t="s">
         <v>1099</v>
       </c>
-      <c r="F12" s="249" t="s">
+      <c r="G12" s="249" t="s">
         <v>1100</v>
       </c>
-      <c r="G12" s="249" t="s">
+      <c r="H12" s="249" t="s">
         <v>1101</v>
-      </c>
-      <c r="H12" s="249" t="s">
-        <v>1102</v>
       </c>
     </row>
     <row r="13" spans="3:8" x14ac:dyDescent="0.25">
@@ -36295,19 +36322,19 @@
         <v>7</v>
       </c>
       <c r="D13" s="295" t="s">
+        <v>1102</v>
+      </c>
+      <c r="E13" s="249" t="s">
         <v>1103</v>
       </c>
-      <c r="E13" s="249" t="s">
+      <c r="F13" s="249" t="s">
         <v>1104</v>
       </c>
-      <c r="F13" s="249" t="s">
+      <c r="G13" s="249" t="s">
         <v>1105</v>
       </c>
-      <c r="G13" s="249" t="s">
+      <c r="H13" s="249" t="s">
         <v>1106</v>
-      </c>
-      <c r="H13" s="249" t="s">
-        <v>1107</v>
       </c>
     </row>
     <row r="14" spans="3:8" x14ac:dyDescent="0.25">
@@ -36315,16 +36342,16 @@
         <v>8</v>
       </c>
       <c r="D14" s="295" t="s">
+        <v>1107</v>
+      </c>
+      <c r="E14" s="249" t="s">
         <v>1108</v>
       </c>
-      <c r="E14" s="249" t="s">
+      <c r="F14" s="249" t="s">
         <v>1109</v>
       </c>
-      <c r="F14" s="249" t="s">
+      <c r="G14" s="249" t="s">
         <v>1110</v>
-      </c>
-      <c r="G14" s="249" t="s">
-        <v>1111</v>
       </c>
       <c r="H14" s="249" t="e">
         <v>#N/A</v>
@@ -36338,13 +36365,13 @@
         <v>1</v>
       </c>
       <c r="E15" s="249" t="s">
+        <v>1111</v>
+      </c>
+      <c r="F15" s="249" t="s">
         <v>1112</v>
       </c>
-      <c r="F15" s="249" t="s">
+      <c r="G15" s="249" t="s">
         <v>1113</v>
-      </c>
-      <c r="G15" s="249" t="s">
-        <v>1114</v>
       </c>
       <c r="H15" s="249" t="b">
         <v>1</v>
@@ -36358,13 +36385,13 @@
         <v>0</v>
       </c>
       <c r="E16" s="249" t="s">
+        <v>1114</v>
+      </c>
+      <c r="F16" s="249" t="s">
         <v>1115</v>
       </c>
-      <c r="F16" s="249" t="s">
-        <v>1116</v>
-      </c>
       <c r="G16" s="249" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="H16" s="249" t="b">
         <v>0</v>
@@ -36375,16 +36402,16 @@
         <v>11</v>
       </c>
       <c r="D17" s="296" t="s">
+        <v>1116</v>
+      </c>
+      <c r="E17" s="267" t="s">
         <v>1117</v>
       </c>
-      <c r="E17" s="267" t="s">
+      <c r="F17" s="267" t="s">
         <v>1118</v>
       </c>
-      <c r="F17" s="267" t="s">
+      <c r="G17" s="267" t="s">
         <v>1119</v>
-      </c>
-      <c r="G17" s="267" t="s">
-        <v>1120</v>
       </c>
       <c r="H17" s="267" t="b">
         <v>0</v>
@@ -36395,16 +36422,16 @@
         <v>12</v>
       </c>
       <c r="D18" s="296" t="s">
+        <v>1120</v>
+      </c>
+      <c r="E18" s="267" t="s">
         <v>1121</v>
       </c>
-      <c r="E18" s="267" t="s">
+      <c r="F18" s="267" t="s">
         <v>1122</v>
       </c>
-      <c r="F18" s="267" t="s">
+      <c r="G18" s="267" t="s">
         <v>1123</v>
-      </c>
-      <c r="G18" s="267" t="s">
-        <v>1124</v>
       </c>
       <c r="H18" s="267" t="b">
         <v>0</v>
@@ -36415,16 +36442,16 @@
         <v>13</v>
       </c>
       <c r="D19" s="296" t="s">
+        <v>1124</v>
+      </c>
+      <c r="E19" s="267" t="s">
         <v>1125</v>
       </c>
-      <c r="E19" s="267" t="s">
+      <c r="F19" s="267" t="s">
         <v>1126</v>
       </c>
-      <c r="F19" s="267" t="s">
+      <c r="G19" s="267" t="s">
         <v>1127</v>
-      </c>
-      <c r="G19" s="267" t="s">
-        <v>1128</v>
       </c>
       <c r="H19" s="267" t="b">
         <v>1</v>
@@ -36435,16 +36462,16 @@
         <v>14</v>
       </c>
       <c r="D20" s="297" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E20" s="264" t="s">
         <v>1129</v>
       </c>
-      <c r="E20" s="264" t="s">
+      <c r="F20" s="264" t="s">
         <v>1130</v>
       </c>
-      <c r="F20" s="264" t="s">
+      <c r="G20" s="264" t="s">
         <v>1131</v>
-      </c>
-      <c r="G20" s="264" t="s">
-        <v>1132</v>
       </c>
       <c r="H20" s="264" t="b">
         <v>0</v>
@@ -36455,16 +36482,16 @@
         <v>15</v>
       </c>
       <c r="D21" s="297" t="s">
+        <v>1132</v>
+      </c>
+      <c r="E21" s="264" t="s">
         <v>1133</v>
       </c>
-      <c r="E21" s="264" t="s">
+      <c r="F21" s="264" t="s">
         <v>1134</v>
       </c>
-      <c r="F21" s="264" t="s">
+      <c r="G21" s="264" t="s">
         <v>1135</v>
-      </c>
-      <c r="G21" s="264" t="s">
-        <v>1136</v>
       </c>
       <c r="H21" s="264" t="b">
         <v>0</v>
@@ -36475,16 +36502,16 @@
         <v>16</v>
       </c>
       <c r="D22" s="298" t="s">
+        <v>1136</v>
+      </c>
+      <c r="E22" s="279" t="s">
         <v>1137</v>
       </c>
-      <c r="E22" s="279" t="s">
+      <c r="F22" s="279" t="s">
         <v>1138</v>
       </c>
-      <c r="F22" s="279" t="s">
+      <c r="G22" s="279" t="s">
         <v>1139</v>
-      </c>
-      <c r="G22" s="279" t="s">
-        <v>1140</v>
       </c>
       <c r="H22" s="279" t="b">
         <v>0</v>
@@ -36495,16 +36522,16 @@
         <v>17</v>
       </c>
       <c r="D23" s="299" t="s">
+        <v>1140</v>
+      </c>
+      <c r="E23" s="243" t="s">
         <v>1141</v>
       </c>
-      <c r="E23" s="243" t="s">
+      <c r="F23" s="243" t="s">
         <v>1142</v>
       </c>
-      <c r="F23" s="243" t="s">
+      <c r="G23" s="243" t="s">
         <v>1143</v>
-      </c>
-      <c r="G23" s="243" t="s">
-        <v>1144</v>
       </c>
       <c r="H23" s="243" t="b">
         <v>0</v>
@@ -36515,16 +36542,16 @@
         <v>18</v>
       </c>
       <c r="D24" s="299" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E24" s="243" t="s">
         <v>1145</v>
       </c>
-      <c r="E24" s="243" t="s">
+      <c r="F24" s="243" t="s">
         <v>1146</v>
       </c>
-      <c r="F24" s="243" t="s">
+      <c r="G24" s="243" t="s">
         <v>1147</v>
-      </c>
-      <c r="G24" s="243" t="s">
-        <v>1148</v>
       </c>
       <c r="H24" s="243" t="b">
         <v>0</v>
@@ -36535,16 +36562,16 @@
         <v>19</v>
       </c>
       <c r="D25" s="300" t="s">
+        <v>1148</v>
+      </c>
+      <c r="E25" s="258" t="s">
         <v>1149</v>
       </c>
-      <c r="E25" s="258" t="s">
+      <c r="F25" s="258" t="s">
         <v>1150</v>
       </c>
-      <c r="F25" s="258" t="s">
+      <c r="G25" s="258" t="s">
         <v>1151</v>
-      </c>
-      <c r="G25" s="258" t="s">
-        <v>1152</v>
       </c>
       <c r="H25" s="258" t="b">
         <v>1</v>
@@ -36555,19 +36582,239 @@
         <v>20</v>
       </c>
       <c r="D26" s="300" t="s">
+        <v>1152</v>
+      </c>
+      <c r="E26" s="258" t="s">
         <v>1153</v>
       </c>
-      <c r="E26" s="258" t="s">
+      <c r="F26" s="258" t="s">
         <v>1154</v>
       </c>
-      <c r="F26" s="258" t="s">
+      <c r="G26" s="258" t="s">
         <v>1155</v>
       </c>
-      <c r="G26" s="258" t="s">
+      <c r="H26" s="258" t="s">
         <v>1156</v>
       </c>
-      <c r="H26" s="258" t="s">
-        <v>1157</v>
+    </row>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C30" s="239" t="s">
+        <v>559</v>
+      </c>
+      <c r="D30" s="239" t="s">
+        <v>560</v>
+      </c>
+      <c r="E30" s="239" t="s">
+        <v>561</v>
+      </c>
+      <c r="F30" s="239" t="s">
+        <v>645</v>
+      </c>
+      <c r="G30" s="239" t="s">
+        <v>562</v>
+      </c>
+      <c r="H30" s="239" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C31" s="249">
+        <v>3</v>
+      </c>
+      <c r="D31" s="295" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E31" s="249" t="s">
+        <v>1086</v>
+      </c>
+      <c r="F31" s="249" t="s">
+        <v>1087</v>
+      </c>
+      <c r="G31" s="249" t="s">
+        <v>1088</v>
+      </c>
+      <c r="H31" s="249" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C32" s="249">
+        <v>4</v>
+      </c>
+      <c r="D32" s="295" t="s">
+        <v>1089</v>
+      </c>
+      <c r="E32" s="249" t="s">
+        <v>1090</v>
+      </c>
+      <c r="F32" s="249" t="s">
+        <v>1091</v>
+      </c>
+      <c r="G32" s="249" t="s">
+        <v>1092</v>
+      </c>
+      <c r="H32" s="249" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C33" s="249">
+        <v>5</v>
+      </c>
+      <c r="D33" s="295" t="s">
+        <v>1093</v>
+      </c>
+      <c r="E33" s="249" t="s">
+        <v>1094</v>
+      </c>
+      <c r="F33" s="249" t="s">
+        <v>1095</v>
+      </c>
+      <c r="G33" s="249" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H33" s="249" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C34" s="249">
+        <v>6</v>
+      </c>
+      <c r="D34" s="295" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E34" s="249" t="s">
+        <v>1098</v>
+      </c>
+      <c r="F34" s="249" t="s">
+        <v>1099</v>
+      </c>
+      <c r="G34" s="249" t="s">
+        <v>1100</v>
+      </c>
+      <c r="H34" s="249" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="35" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C35" s="249">
+        <v>7</v>
+      </c>
+      <c r="D35" s="295" t="s">
+        <v>1102</v>
+      </c>
+      <c r="E35" s="249" t="s">
+        <v>1103</v>
+      </c>
+      <c r="F35" s="249" t="s">
+        <v>1104</v>
+      </c>
+      <c r="G35" s="249" t="s">
+        <v>1105</v>
+      </c>
+      <c r="H35" s="249" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="36" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C36" s="249">
+        <v>8</v>
+      </c>
+      <c r="D36" s="295" t="s">
+        <v>1107</v>
+      </c>
+      <c r="E36" s="249" t="s">
+        <v>1108</v>
+      </c>
+      <c r="F36" s="249" t="s">
+        <v>1109</v>
+      </c>
+      <c r="G36" s="249" t="s">
+        <v>1110</v>
+      </c>
+      <c r="H36" s="249" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="37" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C37" s="249">
+        <v>9</v>
+      </c>
+      <c r="D37" s="295" t="b">
+        <v>1</v>
+      </c>
+      <c r="E37" s="249" t="s">
+        <v>1111</v>
+      </c>
+      <c r="F37" s="249" t="s">
+        <v>1112</v>
+      </c>
+      <c r="G37" s="249" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H37" s="249" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C38" s="249">
+        <v>10</v>
+      </c>
+      <c r="D38" s="295" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" s="249" t="s">
+        <v>1114</v>
+      </c>
+      <c r="F38" s="249" t="s">
+        <v>1115</v>
+      </c>
+      <c r="G38" s="249" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H38" s="249" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C39" s="249">
+        <v>9</v>
+      </c>
+      <c r="D39" s="295" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E39" s="249" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F39" s="249" t="s">
+        <v>1206</v>
+      </c>
+      <c r="G39" s="249" t="s">
+        <v>1207</v>
+      </c>
+      <c r="H39" s="249" t="s">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="40" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C40" s="249">
+        <v>10</v>
+      </c>
+      <c r="D40" s="295" t="s">
+        <v>1209</v>
+      </c>
+      <c r="E40" s="249" t="s">
+        <v>1210</v>
+      </c>
+      <c r="F40" s="249" t="s">
+        <v>1211</v>
+      </c>
+      <c r="G40" s="249" t="s">
+        <v>1212</v>
+      </c>
+      <c r="H40" s="249" t="s">
+        <v>1213</v>
       </c>
     </row>
   </sheetData>
@@ -36597,27 +36844,27 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B2" s="334" t="s">
+      <c r="B2" s="335" t="s">
         <v>553</v>
       </c>
-      <c r="C2" s="335"/>
-      <c r="D2" s="335"/>
-      <c r="E2" s="336"/>
-      <c r="F2" s="318">
+      <c r="C2" s="336"/>
+      <c r="D2" s="336"/>
+      <c r="E2" s="337"/>
+      <c r="F2" s="319">
         <v>500</v>
       </c>
-      <c r="G2" s="337"/>
-      <c r="H2" s="337"/>
-      <c r="I2" s="337"/>
-      <c r="J2" s="337"/>
-      <c r="K2" s="337"/>
+      <c r="G2" s="338"/>
+      <c r="H2" s="338"/>
+      <c r="I2" s="338"/>
+      <c r="J2" s="338"/>
+      <c r="K2" s="338"/>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="167" t="s">
         <v>901</v>
       </c>
       <c r="C3" s="137" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D3" s="137" t="s">
         <v>461</v>
@@ -36629,7 +36876,7 @@
         <v>463</v>
       </c>
       <c r="G3" s="137" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="H3" s="137" t="s">
         <v>464</v>
@@ -36647,31 +36894,31 @@
         <v>533</v>
       </c>
       <c r="M3" s="138" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="N3" s="138" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="O3" s="138" t="s">
+        <v>1200</v>
+      </c>
+      <c r="P3" s="138" t="s">
+        <v>1202</v>
+      </c>
+      <c r="Q3" s="138" t="s">
         <v>1201</v>
       </c>
-      <c r="P3" s="138" t="s">
-        <v>1203</v>
-      </c>
-      <c r="Q3" s="138" t="s">
-        <v>1202</v>
-      </c>
       <c r="S3" s="137" t="s">
+        <v>1163</v>
+      </c>
+      <c r="T3" s="137" t="s">
         <v>1164</v>
       </c>
-      <c r="T3" s="137" t="s">
+      <c r="U3" s="137" t="s">
         <v>1165</v>
       </c>
-      <c r="U3" s="137" t="s">
+      <c r="V3" s="137" t="s">
         <v>1166</v>
-      </c>
-      <c r="V3" s="137" t="s">
-        <v>1167</v>
       </c>
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.25">
@@ -36732,16 +36979,16 @@
         <v>Below Average</v>
       </c>
       <c r="S4" s="105" t="s">
+        <v>1167</v>
+      </c>
+      <c r="T4" s="105" t="s">
         <v>1168</v>
-      </c>
-      <c r="T4" s="105" t="s">
-        <v>1169</v>
       </c>
       <c r="U4" s="105">
         <v>4</v>
       </c>
       <c r="V4" s="105" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
@@ -36802,16 +37049,16 @@
         <v>Fair</v>
       </c>
       <c r="S5" s="105" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="T5" s="105" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="U5" s="105">
         <v>4</v>
       </c>
       <c r="V5" s="105" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
@@ -36872,16 +37119,16 @@
         <v>Very Good</v>
       </c>
       <c r="S6" s="105" t="s">
+        <v>1172</v>
+      </c>
+      <c r="T6" s="105" t="s">
         <v>1173</v>
-      </c>
-      <c r="T6" s="105" t="s">
-        <v>1174</v>
       </c>
       <c r="U6" s="105">
         <v>3.67</v>
       </c>
       <c r="V6" s="105" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
@@ -36942,16 +37189,16 @@
         <v>Passed Non-credit</v>
       </c>
       <c r="S7" s="105" t="s">
+        <v>1175</v>
+      </c>
+      <c r="T7" s="105" t="s">
         <v>1176</v>
-      </c>
-      <c r="T7" s="105" t="s">
-        <v>1177</v>
       </c>
       <c r="U7" s="105">
         <v>3.33</v>
       </c>
       <c r="V7" s="105" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -37012,16 +37259,16 @@
         <v>Fair</v>
       </c>
       <c r="S8" s="105" t="s">
+        <v>1178</v>
+      </c>
+      <c r="T8" s="105" t="s">
         <v>1179</v>
-      </c>
-      <c r="T8" s="105" t="s">
-        <v>1180</v>
       </c>
       <c r="U8" s="105">
         <v>3</v>
       </c>
       <c r="V8" s="105" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -37082,16 +37329,16 @@
         <v>Fair</v>
       </c>
       <c r="S9" s="105" t="s">
+        <v>1181</v>
+      </c>
+      <c r="T9" s="105" t="s">
         <v>1182</v>
-      </c>
-      <c r="T9" s="105" t="s">
-        <v>1183</v>
       </c>
       <c r="U9" s="105">
         <v>2.67</v>
       </c>
       <c r="V9" s="105" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -37152,16 +37399,16 @@
         <v>Average</v>
       </c>
       <c r="S10" s="105" t="s">
+        <v>1184</v>
+      </c>
+      <c r="T10" s="105" t="s">
         <v>1185</v>
-      </c>
-      <c r="T10" s="105" t="s">
-        <v>1186</v>
       </c>
       <c r="U10" s="105">
         <v>2.33</v>
       </c>
       <c r="V10" s="105" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -37222,16 +37469,16 @@
         <v>Good</v>
       </c>
       <c r="S11" s="105" t="s">
+        <v>1187</v>
+      </c>
+      <c r="T11" s="105" t="s">
         <v>1188</v>
-      </c>
-      <c r="T11" s="105" t="s">
-        <v>1189</v>
       </c>
       <c r="U11" s="105">
         <v>2</v>
       </c>
       <c r="V11" s="105" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -37292,16 +37539,16 @@
         <v>Excellent</v>
       </c>
       <c r="S12" s="105" t="s">
+        <v>1190</v>
+      </c>
+      <c r="T12" s="105" t="s">
         <v>1191</v>
-      </c>
-      <c r="T12" s="105" t="s">
-        <v>1192</v>
       </c>
       <c r="U12" s="105">
         <v>1.67</v>
       </c>
       <c r="V12" s="105" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -37362,16 +37609,16 @@
         <v>Good</v>
       </c>
       <c r="S13" s="105" t="s">
+        <v>1192</v>
+      </c>
+      <c r="T13" s="105" t="s">
         <v>1193</v>
       </c>
-      <c r="T13" s="105" t="s">
+      <c r="U13" s="105" t="s">
         <v>1194</v>
       </c>
-      <c r="U13" s="105" t="s">
+      <c r="V13" s="105" t="s">
         <v>1195</v>
-      </c>
-      <c r="V13" s="105" t="s">
-        <v>1196</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -37432,16 +37679,16 @@
         <v>Fair</v>
       </c>
       <c r="S14" s="105" t="s">
+        <v>1196</v>
+      </c>
+      <c r="T14" s="105" t="s">
         <v>1197</v>
-      </c>
-      <c r="T14" s="105" t="s">
-        <v>1198</v>
       </c>
       <c r="U14" s="105">
         <v>0</v>
       </c>
       <c r="V14" s="105" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -37681,25 +37928,25 @@
         <v>901</v>
       </c>
       <c r="C23" s="137" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D23" s="137" t="s">
         <v>45</v>
       </c>
       <c r="E23" s="137" t="s">
+        <v>1158</v>
+      </c>
+      <c r="F23" s="137" t="s">
         <v>1159</v>
       </c>
-      <c r="F23" s="137" t="s">
+      <c r="G23" s="137" t="s">
+        <v>1085</v>
+      </c>
+      <c r="H23" s="137" t="s">
+        <v>1089</v>
+      </c>
+      <c r="I23" s="137" t="s">
         <v>1160</v>
-      </c>
-      <c r="G23" s="137" t="s">
-        <v>1086</v>
-      </c>
-      <c r="H23" s="137" t="s">
-        <v>1090</v>
-      </c>
-      <c r="I23" s="137" t="s">
-        <v>1161</v>
       </c>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.25">
@@ -37712,7 +37959,7 @@
       <c r="D24" s="105">
         <v>46829</v>
       </c>
-      <c r="E24" s="338">
+      <c r="E24" s="301">
         <f>IF(D24&gt;=70000,5,IF(D24&gt;=60000,4,IF(D24&gt;=50000,3,IF(D24&gt;=40000,2,1))))</f>
         <v>2</v>
       </c>
@@ -37721,19 +37968,19 @@
         <v>No Bonus</v>
       </c>
       <c r="G24" s="105" t="b">
-        <f>AND(D24&gt;=50000,E24&gt;=3)</f>
+        <f t="shared" ref="G24:G38" si="3">AND(D24&gt;=50000,E24&gt;=3)</f>
         <v>0</v>
       </c>
       <c r="H24" s="105" t="b">
-        <f>OR(D24&gt;=50000,E24&gt;=3)</f>
+        <f t="shared" ref="H24:H38" si="4">OR(D24&gt;=50000,E24&gt;=3)</f>
         <v>0</v>
       </c>
       <c r="I24" s="105" t="str">
-        <f>IF(OR(D24&gt;=50000,E24&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" ref="I24:I38" si="5">IF(OR(D24&gt;=50000,E24&gt;=3),"Bonus Eligible","No Bonus")</f>
         <v>No Bonus</v>
       </c>
       <c r="Q24" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.25">
@@ -37746,24 +37993,24 @@
       <c r="D25" s="105">
         <v>52917</v>
       </c>
-      <c r="E25" s="338">
-        <f t="shared" ref="E25:E38" si="3">IF(D25&gt;=70000,5,IF(D25&gt;=60000,4,IF(D25&gt;=50000,3,IF(D25&gt;=40000,2,1))))</f>
+      <c r="E25" s="301">
+        <f t="shared" ref="E25:E38" si="6">IF(D25&gt;=70000,5,IF(D25&gt;=60000,4,IF(D25&gt;=50000,3,IF(D25&gt;=40000,2,1))))</f>
         <v>3</v>
       </c>
       <c r="F25" s="105" t="str">
-        <f t="shared" ref="F25:F38" si="4">IF(AND(D25&gt;=50000,E25&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" ref="F25:F38" si="7">IF(AND(D25&gt;=50000,E25&gt;=3),"Bonus Eligible","No Bonus")</f>
         <v>Bonus Eligible</v>
       </c>
       <c r="G25" s="105" t="b">
-        <f>AND(D25&gt;=50000,E25&gt;=3)</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H25" s="105" t="b">
-        <f>OR(D25&gt;=50000,E25&gt;=3)</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I25" s="105" t="str">
-        <f>IF(OR(D25&gt;=50000,E25&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37777,24 +38024,24 @@
       <c r="D26" s="105">
         <v>66037</v>
       </c>
-      <c r="E26" s="338">
+      <c r="E26" s="301">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="F26" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G26" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="F26" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H26" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G26" s="105" t="b">
-        <f>AND(D26&gt;=50000,E26&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H26" s="105" t="b">
-        <f>OR(D26&gt;=50000,E26&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I26" s="105" t="str">
-        <f>IF(OR(D26&gt;=50000,E26&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37808,24 +38055,24 @@
       <c r="D27" s="105">
         <v>51623</v>
       </c>
-      <c r="E27" s="338">
+      <c r="E27" s="301">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="F27" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G27" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="F27" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H27" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G27" s="105" t="b">
-        <f>AND(D27&gt;=50000,E27&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H27" s="105" t="b">
-        <f>OR(D27&gt;=50000,E27&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I27" s="105" t="str">
-        <f>IF(OR(D27&gt;=50000,E27&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37839,24 +38086,24 @@
       <c r="D28" s="105">
         <v>58370</v>
       </c>
-      <c r="E28" s="338">
+      <c r="E28" s="301">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="F28" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G28" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="F28" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H28" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G28" s="105" t="b">
-        <f>AND(D28&gt;=50000,E28&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H28" s="105" t="b">
-        <f>OR(D28&gt;=50000,E28&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I28" s="105" t="str">
-        <f>IF(OR(D28&gt;=50000,E28&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37870,24 +38117,24 @@
       <c r="D29" s="105">
         <v>48375</v>
       </c>
-      <c r="E29" s="338">
+      <c r="E29" s="301">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="F29" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="G29" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="F29" s="105" t="str">
+        <v>0</v>
+      </c>
+      <c r="H29" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>No Bonus</v>
-      </c>
-      <c r="G29" s="105" t="b">
-        <f>AND(D29&gt;=50000,E29&gt;=3)</f>
         <v>0</v>
       </c>
-      <c r="H29" s="105" t="b">
-        <f>OR(D29&gt;=50000,E29&gt;=3)</f>
-        <v>0</v>
-      </c>
       <c r="I29" s="105" t="str">
-        <f>IF(OR(D29&gt;=50000,E29&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>No Bonus</v>
       </c>
     </row>
@@ -37901,24 +38148,24 @@
       <c r="D30" s="105">
         <v>65352</v>
       </c>
-      <c r="E30" s="338">
+      <c r="E30" s="301">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="F30" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G30" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="F30" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H30" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G30" s="105" t="b">
-        <f>AND(D30&gt;=50000,E30&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H30" s="105" t="b">
-        <f>OR(D30&gt;=50000,E30&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I30" s="105" t="str">
-        <f>IF(OR(D30&gt;=50000,E30&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37932,24 +38179,24 @@
       <c r="D31" s="105">
         <v>69904</v>
       </c>
-      <c r="E31" s="338">
+      <c r="E31" s="301">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="F31" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G31" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="F31" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H31" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G31" s="105" t="b">
-        <f>AND(D31&gt;=50000,E31&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H31" s="105" t="b">
-        <f>OR(D31&gt;=50000,E31&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I31" s="105" t="str">
-        <f>IF(OR(D31&gt;=50000,E31&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37963,24 +38210,24 @@
       <c r="D32" s="105">
         <v>76618</v>
       </c>
-      <c r="E32" s="338">
+      <c r="E32" s="301">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="F32" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G32" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="F32" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H32" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G32" s="105" t="b">
-        <f>AND(D32&gt;=50000,E32&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H32" s="105" t="b">
-        <f>OR(D32&gt;=50000,E32&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I32" s="105" t="str">
-        <f>IF(OR(D32&gt;=50000,E32&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -37994,24 +38241,24 @@
       <c r="D33" s="105">
         <v>65398</v>
       </c>
-      <c r="E33" s="338">
+      <c r="E33" s="301">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="F33" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G33" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="F33" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H33" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G33" s="105" t="b">
-        <f>AND(D33&gt;=50000,E33&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H33" s="105" t="b">
-        <f>OR(D33&gt;=50000,E33&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I33" s="105" t="str">
-        <f>IF(OR(D33&gt;=50000,E33&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -38025,24 +38272,24 @@
       <c r="D34" s="105">
         <v>73129</v>
       </c>
-      <c r="E34" s="338">
+      <c r="E34" s="301">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="F34" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G34" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="F34" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H34" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G34" s="105" t="b">
-        <f>AND(D34&gt;=50000,E34&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H34" s="105" t="b">
-        <f>OR(D34&gt;=50000,E34&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I34" s="105" t="str">
-        <f>IF(OR(D34&gt;=50000,E34&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -38056,24 +38303,24 @@
       <c r="D35" s="105">
         <v>45692</v>
       </c>
-      <c r="E35" s="338">
+      <c r="E35" s="301">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="F35" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="G35" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="F35" s="105" t="str">
+        <v>0</v>
+      </c>
+      <c r="H35" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>No Bonus</v>
-      </c>
-      <c r="G35" s="105" t="b">
-        <f>AND(D35&gt;=50000,E35&gt;=3)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="105" t="b">
-        <f>OR(D35&gt;=50000,E35&gt;=3)</f>
-        <v>0</v>
-      </c>
       <c r="I35" s="105" t="str">
-        <f>IF(OR(D35&gt;=50000,E35&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>No Bonus</v>
       </c>
     </row>
@@ -38087,24 +38334,24 @@
       <c r="D36" s="105">
         <v>64141</v>
       </c>
-      <c r="E36" s="338">
+      <c r="E36" s="301">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="F36" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G36" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="F36" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H36" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G36" s="105" t="b">
-        <f>AND(D36&gt;=50000,E36&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H36" s="105" t="b">
-        <f>OR(D36&gt;=50000,E36&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I36" s="105" t="str">
-        <f>IF(OR(D36&gt;=50000,E36&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -38118,24 +38365,24 @@
       <c r="D37" s="105">
         <v>60639</v>
       </c>
-      <c r="E37" s="338">
+      <c r="E37" s="301">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="F37" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>Bonus Eligible</v>
+      </c>
+      <c r="G37" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="F37" s="105" t="str">
+        <v>1</v>
+      </c>
+      <c r="H37" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>Bonus Eligible</v>
-      </c>
-      <c r="G37" s="105" t="b">
-        <f>AND(D37&gt;=50000,E37&gt;=3)</f>
         <v>1</v>
       </c>
-      <c r="H37" s="105" t="b">
-        <f>OR(D37&gt;=50000,E37&gt;=3)</f>
-        <v>1</v>
-      </c>
       <c r="I37" s="105" t="str">
-        <f>IF(OR(D37&gt;=50000,E37&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>Bonus Eligible</v>
       </c>
     </row>
@@ -38149,24 +38396,24 @@
       <c r="D38" s="105">
         <v>24501</v>
       </c>
-      <c r="E38" s="338">
+      <c r="E38" s="301">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="F38" s="105" t="str">
+        <f t="shared" si="7"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="G38" s="105" t="b">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="F38" s="105" t="str">
+        <v>0</v>
+      </c>
+      <c r="H38" s="105" t="b">
         <f t="shared" si="4"/>
-        <v>No Bonus</v>
-      </c>
-      <c r="G38" s="105" t="b">
-        <f>AND(D38&gt;=50000,E38&gt;=3)</f>
         <v>0</v>
       </c>
-      <c r="H38" s="105" t="b">
-        <f>OR(D38&gt;=50000,E38&gt;=3)</f>
-        <v>0</v>
-      </c>
       <c r="I38" s="105" t="str">
-        <f>IF(OR(D38&gt;=50000,E38&gt;=3),"Bonus Eligible","No Bonus")</f>
+        <f t="shared" si="5"/>
         <v>No Bonus</v>
       </c>
     </row>
@@ -38228,11 +38475,11 @@
       </c>
       <c r="D2" s="25">
         <f t="shared" ref="C2:F15" ca="1" si="0">RANDBETWEEN(0,100)</f>
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="E2" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="28">
@@ -38254,16 +38501,16 @@
       </c>
       <c r="C3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>92</v>
       </c>
       <c r="D3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E3" s="25"/>
       <c r="F3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G3" s="28">
         <f t="shared" ref="G3:G15" ca="1" si="1">COUNT(C3:F3)</f>
@@ -38285,11 +38532,11 @@
       <c r="C4" s="25"/>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="28">
@@ -38311,16 +38558,16 @@
       </c>
       <c r="C5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="D5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <v>92</v>
       </c>
       <c r="E5" s="25"/>
       <c r="F5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="G5" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38341,16 +38588,16 @@
       </c>
       <c r="C6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="E6" s="25"/>
       <c r="F6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="G6" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38372,15 +38619,15 @@
       <c r="C7" s="25"/>
       <c r="D7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="E7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="F7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="G7" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38401,7 +38648,7 @@
       </c>
       <c r="C8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>468</v>
@@ -38411,7 +38658,7 @@
       </c>
       <c r="F8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="G8" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38432,19 +38679,19 @@
       </c>
       <c r="C9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="G9" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38465,12 +38712,12 @@
       </c>
       <c r="C10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="D10" s="25"/>
       <c r="E10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="F10" s="25"/>
       <c r="G10" s="28">
@@ -38492,19 +38739,19 @@
       </c>
       <c r="C11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="E11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="F11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="G11" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38525,15 +38772,15 @@
       </c>
       <c r="C12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="D12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="E12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>12</v>
       </c>
       <c r="F12" s="25"/>
       <c r="G12" s="28">
@@ -38555,16 +38802,16 @@
       </c>
       <c r="C13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="G13" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38585,18 +38832,18 @@
       </c>
       <c r="C14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>468</v>
       </c>
       <c r="F14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="G14" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -38621,7 +38868,7 @@
       <c r="D15" s="27"/>
       <c r="E15" s="27">
         <f t="shared" ca="1" si="0"/>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>468</v>
@@ -43058,54 +43305,54 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E51">
-    <cfRule type="cellIs" dxfId="43" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="44" operator="equal">
       <formula>20000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="45" operator="between">
+    <cfRule type="cellIs" dxfId="58" priority="45" operator="between">
       <formula>50000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="46" operator="between">
+    <cfRule type="cellIs" dxfId="57" priority="46" operator="between">
       <formula>"Rs. 65,984"</formula>
       <formula>"Rs. 121,395"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="47" operator="lessThan">
+    <cfRule type="cellIs" dxfId="56" priority="47" operator="lessThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="48" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="55" priority="48" operator="greaterThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="49" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="54" priority="49" operator="greaterThan">
       <formula>"Rs. 93,689"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B53">
-    <cfRule type="containsText" dxfId="37" priority="43" operator="containsText" text="Ayesha khan">
+    <cfRule type="containsText" dxfId="53" priority="43" operator="containsText" text="Ayesha khan">
       <formula>NOT(ISERROR(SEARCH("Ayesha khan",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A53">
-    <cfRule type="timePeriod" dxfId="36" priority="41" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="52" priority="41" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="35" priority="42" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="51" priority="42" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A53">
-    <cfRule type="timePeriod" dxfId="34" priority="38" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="50" priority="38" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A2,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A2,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="33" priority="39" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="49" priority="39" timePeriod="yesterday">
       <formula>FLOOR(A2,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="32" priority="40" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="48" priority="40" timePeriod="today">
       <formula>FLOOR(A2,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="uniqueValues" dxfId="31" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="37"/>
+    <cfRule type="uniqueValues" dxfId="47" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E55:E105">
     <cfRule type="dataBar" priority="18">
@@ -45321,13 +45568,13 @@
     </row>
     <row r="58" spans="3:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C59" s="301" t="s">
+      <c r="C59" s="302" t="s">
         <v>528</v>
       </c>
-      <c r="D59" s="302"/>
-      <c r="E59" s="302"/>
-      <c r="F59" s="302"/>
-      <c r="G59" s="302"/>
+      <c r="D59" s="303"/>
+      <c r="E59" s="303"/>
+      <c r="F59" s="303"/>
+      <c r="G59" s="303"/>
       <c r="H59" s="88"/>
     </row>
     <row r="60" spans="3:8" x14ac:dyDescent="0.25">
@@ -50627,40 +50874,40 @@
     </row>
     <row r="168" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="169" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A169" s="303" t="s">
+      <c r="A169" s="304" t="s">
         <v>534</v>
       </c>
-      <c r="B169" s="304"/>
-      <c r="C169" s="304"/>
-      <c r="D169" s="304"/>
-      <c r="E169" s="304"/>
-      <c r="F169" s="304"/>
-      <c r="G169" s="304"/>
-      <c r="H169" s="304"/>
-      <c r="I169" s="304"/>
-      <c r="J169" s="304"/>
-      <c r="K169" s="304"/>
-      <c r="L169" s="304"/>
-      <c r="M169" s="304"/>
-      <c r="N169" s="304"/>
-      <c r="O169" s="305"/>
+      <c r="B169" s="305"/>
+      <c r="C169" s="305"/>
+      <c r="D169" s="305"/>
+      <c r="E169" s="305"/>
+      <c r="F169" s="305"/>
+      <c r="G169" s="305"/>
+      <c r="H169" s="305"/>
+      <c r="I169" s="305"/>
+      <c r="J169" s="305"/>
+      <c r="K169" s="305"/>
+      <c r="L169" s="305"/>
+      <c r="M169" s="305"/>
+      <c r="N169" s="305"/>
+      <c r="O169" s="306"/>
     </row>
     <row r="170" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="306"/>
-      <c r="B170" s="307"/>
-      <c r="C170" s="307"/>
-      <c r="D170" s="307"/>
-      <c r="E170" s="307"/>
-      <c r="F170" s="307"/>
-      <c r="G170" s="307"/>
-      <c r="H170" s="307"/>
-      <c r="I170" s="307"/>
-      <c r="J170" s="307"/>
-      <c r="K170" s="307"/>
-      <c r="L170" s="307"/>
-      <c r="M170" s="307"/>
-      <c r="N170" s="307"/>
-      <c r="O170" s="308"/>
+      <c r="A170" s="307"/>
+      <c r="B170" s="308"/>
+      <c r="C170" s="308"/>
+      <c r="D170" s="308"/>
+      <c r="E170" s="308"/>
+      <c r="F170" s="308"/>
+      <c r="G170" s="308"/>
+      <c r="H170" s="308"/>
+      <c r="I170" s="308"/>
+      <c r="J170" s="308"/>
+      <c r="K170" s="308"/>
+      <c r="L170" s="308"/>
+      <c r="M170" s="308"/>
+      <c r="N170" s="308"/>
+      <c r="O170" s="309"/>
     </row>
     <row r="171" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A171" s="112"/>

</xml_diff>